<commit_message>
Importados: hoja por titulo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SmQ59SXzFJRTF75F5XCdhw
</commit_message>
<xml_diff>
--- a/ateneo/historial/2026-10/importados_15-10/Importados_por_cliente.xlsx
+++ b/ateneo/historial/2026-10/importados_15-10/Importados_por_cliente.xlsx
@@ -10,10 +10,12 @@
     <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Por cliente" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Sin liquidar" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Por título" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Por cliente'!$A$3:$M$284</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sin liquidar'!$A$3:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Por título'!$A$3:$L$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -13835,4 +13837,2637 @@
   <autoFilter ref="A3:I14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Entregados y liquidados por título · ordenado por entregados</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>ISBN</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Título</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Clientes</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Entregados</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Liquidados</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>% liquidado</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Participación en lo liquidado</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>Devueltos</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>Saldo</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Clientes sin venta del título</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>Pedido Yenny</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="n">
+        <v>747645</v>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>9789500217040</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>DINO, ¿POR QUE ESTAS TRISTE?</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>232</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>1536</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>276</v>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>0.1796875</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>0.02995441719123074</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>1238</v>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>118</v>
+      </c>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t>2240044747</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="n">
+        <v>744141</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>9789500217149</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>100 MENSAJES PARA NIÑOS FELICES</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>1519</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>154</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>0.1013824884792627</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>0.01671369654873019</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>1317</v>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>153</v>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>2240044594</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n">
+        <v>747642</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>9789500217064</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>PEQUEÑOS LIBROS - LITTLE BOOKS</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>227</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>1465</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>242</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>0.1651877133105802</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>0.02626438029086173</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>1206</v>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>124</v>
+      </c>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
+          <t>2240044747</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="n">
+        <v>744139</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>9789500217019</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>HOLA, BEBE. MI MUNDO</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>234</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>1451</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>135</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>0.09303928325292901</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>0.01465161710440634</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>1287</v>
+      </c>
+      <c r="K7" s="8" t="n">
+        <v>146</v>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>2240044592</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n">
+        <v>744140</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>9789500217002</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>HOLA, BEBE. ANIMALES</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>1445</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>124</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>0.08581314878892733</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>0.0134577816366399</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>1292</v>
+      </c>
+      <c r="K8" s="8" t="n">
+        <v>164</v>
+      </c>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>2240044592 / 2240044593</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n">
+        <v>748590</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>9789500217309</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>AQUI ESTOY! DINOSAURITO</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>219</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>0.06853146853146853</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>0.0106359887128283</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>1298</v>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>167</v>
+      </c>
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>2240044767</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>732485</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>9789500215886</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>¡ACA ESTOY! BALLENITA</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>235</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>1428</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>277</v>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>0.1939775910364146</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>0.03006294768830041</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>1119</v>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>2240043597 / 2240044286</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n">
+        <v>741981</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>9789500216807</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>AMIGOS DEL BOSQUE</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>226</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>1424</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>275</v>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>0.1931179775280899</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>0.02984588669416106</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>1099</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>2240044306</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n">
+        <v>747646</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>9789500217026</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>STICKERS MAGICOS DINOSAURIOS</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>224</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>1417</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>277</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>0.1954834156669019</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>0.03006294768830041</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="J12" s="9" t="n">
+        <v>1112</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>113</v>
+      </c>
+      <c r="L12" s="8" t="inlineStr">
+        <is>
+          <t>2240044747</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n">
+        <v>742446</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>9789500216760</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>PEQUEÑOS PASOS: MI MUNDO</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>234</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>1404</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>232</v>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>0.1652421652421652</v>
+      </c>
+      <c r="H13" s="11" t="n">
+        <v>0.02517907532016497</v>
+      </c>
+      <c r="I13" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="J13" s="9" t="n">
+        <v>1142</v>
+      </c>
+      <c r="K13" s="8" t="n">
+        <v>128</v>
+      </c>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>2240044331</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n">
+        <v>742445</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>9789500216777</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>PEQUEÑOS PASOS: MIS ANIMALES</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>226</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>1371</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>214</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>0.1560904449307075</v>
+      </c>
+      <c r="H14" s="11" t="n">
+        <v>0.02322552637291079</v>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="J14" s="9" t="n">
+        <v>1135</v>
+      </c>
+      <c r="K14" s="8" t="n">
+        <v>125</v>
+      </c>
+      <c r="L14" s="8" t="inlineStr">
+        <is>
+          <t>2240044331</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n">
+        <v>750397</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>9789500217552</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>MIS AUTOS DE CARRERA</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>220</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>1364</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>0.04472140762463343</v>
+      </c>
+      <c r="H15" s="11" t="n">
+        <v>0.006620360321250272</v>
+      </c>
+      <c r="I15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="9" t="n">
+        <v>1303</v>
+      </c>
+      <c r="K15" s="8" t="n">
+        <v>185</v>
+      </c>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>2240044948</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n">
+        <v>749100</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>9789500217477</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>PEQUEÑO DRAGON QUE PERDIO SU FUEGO, EL</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>219</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>1346</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="G16" s="10" t="n">
+        <v>0.02897473997028232</v>
+      </c>
+      <c r="H16" s="11" t="n">
+        <v>0.004232689385717386</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J16" s="9" t="n">
+        <v>1305</v>
+      </c>
+      <c r="K16" s="8" t="n">
+        <v>198</v>
+      </c>
+      <c r="L16" s="8" t="inlineStr">
+        <is>
+          <t>2240044947</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n">
+        <v>749098</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>9789500217484</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>PEQUEÑO UNICORNIO QUE PERDIO SU MAGIA, EL</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>218</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>1344</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>0.03794642857142857</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>0.005535055350553505</v>
+      </c>
+      <c r="I17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="9" t="n">
+        <v>1293</v>
+      </c>
+      <c r="K17" s="8" t="n">
+        <v>190</v>
+      </c>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>2240044947</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n">
+        <v>750395</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>9789500217545</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>MIS EXCAVADORAS</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>218</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>1339</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>0.03360716952949962</v>
+      </c>
+      <c r="H18" s="11" t="n">
+        <v>0.004883872368135446</v>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="9" t="n">
+        <v>1294</v>
+      </c>
+      <c r="K18" s="8" t="n">
+        <v>188</v>
+      </c>
+      <c r="L18" s="8" t="inlineStr">
+        <is>
+          <t>2240044948</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n">
+        <v>741979</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>9789500216814</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>AMIGOS DE LA GRANJA</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>220</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>1333</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>307</v>
+      </c>
+      <c r="G19" s="10" t="n">
+        <v>0.2303075768942235</v>
+      </c>
+      <c r="H19" s="11" t="n">
+        <v>0.03331886260039071</v>
+      </c>
+      <c r="I19" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="J19" s="9" t="n">
+        <v>980</v>
+      </c>
+      <c r="K19" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="L19" s="8" t="inlineStr">
+        <is>
+          <t>2240044306</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n">
+        <v>749099</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>9789500217491</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>PEQUEÑO MONO QUE PERDIO SU MIEDO, EL</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>218</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>1322</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="G20" s="10" t="n">
+        <v>0.03857791225416037</v>
+      </c>
+      <c r="H20" s="11" t="n">
+        <v>0.005535055350553505</v>
+      </c>
+      <c r="I20" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>1269</v>
+      </c>
+      <c r="K20" s="8" t="n">
+        <v>188</v>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
+        <is>
+          <t>2240044947</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n">
+        <v>740761</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>9789500216555</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>VAMOS A CONTAR LOS NUMEROS</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>213</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>1320</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>145</v>
+      </c>
+      <c r="G21" s="10" t="n">
+        <v>0.1098484848484848</v>
+      </c>
+      <c r="H21" s="11" t="n">
+        <v>0.0157369220751031</v>
+      </c>
+      <c r="I21" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="J21" s="9" t="n">
+        <v>1117</v>
+      </c>
+      <c r="K21" s="8" t="n">
+        <v>135</v>
+      </c>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t>2240044245</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n">
+        <v>747643</v>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>9789500217057</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>GATITO, ¿POR QUE ESTAS ENOJADO?</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>211</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>1305</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>321</v>
+      </c>
+      <c r="G22" s="10" t="n">
+        <v>0.2459770114942529</v>
+      </c>
+      <c r="H22" s="11" t="n">
+        <v>0.03483828955936618</v>
+      </c>
+      <c r="I22" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="J22" s="9" t="n">
+        <v>973</v>
+      </c>
+      <c r="K22" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="L22" s="8" t="inlineStr">
+        <is>
+          <t>2240044747</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n">
+        <v>751243</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>9789500217682</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>ANIMALES SALVAJES</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>217</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>1301</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>0.004611837048424289</v>
+      </c>
+      <c r="H23" s="11" t="n">
+        <v>0.0006511829824180595</v>
+      </c>
+      <c r="I23" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J23" s="9" t="n">
+        <v>1292</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>213</v>
+      </c>
+      <c r="L23" s="8" t="inlineStr">
+        <is>
+          <t>2240045027</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n">
+        <v>740173</v>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>9789500216517</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>BENJAMIN EN EL JARDIN</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>197</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>1292</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>342</v>
+      </c>
+      <c r="G24" s="10" t="n">
+        <v>0.2647058823529412</v>
+      </c>
+      <c r="H24" s="11" t="n">
+        <v>0.03711742999782939</v>
+      </c>
+      <c r="I24" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="J24" s="9" t="n">
+        <v>929</v>
+      </c>
+      <c r="K24" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="L24" s="8" t="inlineStr">
+        <is>
+          <t>2240044145 / 2240044246</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n">
+        <v>737808</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>9789500216449</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>APRENDO A LEER LAS PALABRAS</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>202</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>1290</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>298</v>
+      </c>
+      <c r="G25" s="10" t="n">
+        <v>0.2310077519379845</v>
+      </c>
+      <c r="H25" s="11" t="n">
+        <v>0.03234208812676362</v>
+      </c>
+      <c r="I25" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="J25" s="9" t="n">
+        <v>905</v>
+      </c>
+      <c r="K25" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="L25" s="8" t="inlineStr">
+        <is>
+          <t>2240044025</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n">
+        <v>751240</v>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>9789500217408</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>MIRA Y DESCUBRE: EL ESPACIO</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>217</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>1290</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J26" s="9" t="n">
+        <v>1287</v>
+      </c>
+      <c r="K26" s="8" t="n">
+        <v>217</v>
+      </c>
+      <c r="L26" s="8" t="inlineStr">
+        <is>
+          <t>2240045047</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n">
+        <v>751241</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>9789500217415</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>MIRA Y DESCUBRE: EL CUERPO HUMANO</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>217</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>1288</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J27" s="9" t="n">
+        <v>1285</v>
+      </c>
+      <c r="K27" s="8" t="n">
+        <v>217</v>
+      </c>
+      <c r="L27" s="8" t="inlineStr">
+        <is>
+          <t>2240045047</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n">
+        <v>740175</v>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>9789500216524</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>RENATA EN LA GRANJA</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>196</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>1283</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>342</v>
+      </c>
+      <c r="G28" s="10" t="n">
+        <v>0.2665627435697584</v>
+      </c>
+      <c r="H28" s="11" t="n">
+        <v>0.03711742999782939</v>
+      </c>
+      <c r="I28" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="J28" s="9" t="n">
+        <v>912</v>
+      </c>
+      <c r="K28" s="8" t="n">
+        <v>71</v>
+      </c>
+      <c r="L28" s="8" t="inlineStr">
+        <is>
+          <t>2240044145 / 2240044246</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n">
+        <v>732486</v>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>9789500215893</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>¡ACA ESTOY! VAQUITA</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>217</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>1282</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>308</v>
+      </c>
+      <c r="G29" s="10" t="n">
+        <v>0.2402496099843994</v>
+      </c>
+      <c r="H29" s="11" t="n">
+        <v>0.03342739309746039</v>
+      </c>
+      <c r="I29" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="J29" s="9" t="n">
+        <v>937</v>
+      </c>
+      <c r="K29" s="8" t="n">
+        <v>82</v>
+      </c>
+      <c r="L29" s="8" t="inlineStr">
+        <is>
+          <t>2240043597 / 2240044286</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n">
+        <v>737452</v>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>9789500216395</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>EXTRAÑO CASO DEL DR. JEKYLL Y MR. HYDE, EL</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>204</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>1271</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>161</v>
+      </c>
+      <c r="G30" s="10" t="n">
+        <v>0.1266719118804091</v>
+      </c>
+      <c r="H30" s="11" t="n">
+        <v>0.01747341002821793</v>
+      </c>
+      <c r="I30" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="J30" s="9" t="n">
+        <v>1052</v>
+      </c>
+      <c r="K30" s="8" t="n">
+        <v>133</v>
+      </c>
+      <c r="L30" s="8" t="inlineStr">
+        <is>
+          <t>2240043984</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n">
+        <v>737041</v>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>9789500216357</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>QUIEN ESTA AHI? EN LA SELVA</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>199</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>1261</v>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>233</v>
+      </c>
+      <c r="G31" s="10" t="n">
+        <v>0.1847739888977002</v>
+      </c>
+      <c r="H31" s="11" t="n">
+        <v>0.02528760581723464</v>
+      </c>
+      <c r="I31" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="J31" s="9" t="n">
+        <v>977</v>
+      </c>
+      <c r="K31" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="L31" s="8" t="inlineStr">
+        <is>
+          <t>2240043968</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n">
+        <v>751242</v>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>9789500217798</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>VAMOS A APRENDER SUMAS Y RESTAS</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>215</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>1257</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" s="9" t="n">
+        <v>1254</v>
+      </c>
+      <c r="K32" s="8" t="n">
+        <v>215</v>
+      </c>
+      <c r="L32" s="8" t="inlineStr">
+        <is>
+          <t>2240045048</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n">
+        <v>747647</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>9789500217033</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>STICKERS MAGICOS: GRANJA</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>204</v>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>1248</v>
+      </c>
+      <c r="F33" s="9" t="n">
+        <v>312</v>
+      </c>
+      <c r="G33" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H33" s="11" t="n">
+        <v>0.03386151508573909</v>
+      </c>
+      <c r="I33" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="J33" s="9" t="n">
+        <v>911</v>
+      </c>
+      <c r="K33" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="L33" s="8" t="inlineStr">
+        <is>
+          <t>2240044747</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n">
+        <v>737882</v>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>9789500216456</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>AUGE Y CAIDA</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>202</v>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>1241</v>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>105</v>
+      </c>
+      <c r="G34" s="10" t="n">
+        <v>0.08460918614020951</v>
+      </c>
+      <c r="H34" s="11" t="n">
+        <v>0.01139570219231604</v>
+      </c>
+      <c r="I34" s="9" t="n">
+        <v>77</v>
+      </c>
+      <c r="J34" s="9" t="n">
+        <v>1062</v>
+      </c>
+      <c r="K34" s="8" t="n">
+        <v>143</v>
+      </c>
+      <c r="L34" s="8" t="inlineStr">
+        <is>
+          <t>2240044057</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n">
+        <v>742443</v>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>9789500216944</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>EXPLOREMOS LA GRANJA</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>220</v>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>1202</v>
+      </c>
+      <c r="F35" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="G35" s="10" t="n">
+        <v>0.07071547420965059</v>
+      </c>
+      <c r="H35" s="11" t="n">
+        <v>0.009225092250922509</v>
+      </c>
+      <c r="I35" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="J35" s="9" t="n">
+        <v>1075</v>
+      </c>
+      <c r="K35" s="8" t="n">
+        <v>163</v>
+      </c>
+      <c r="L35" s="8" t="inlineStr">
+        <is>
+          <t>2240044330</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n">
+        <v>737450</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>9789500216371</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>ARTE DE LA GUERRA, EL</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>191</v>
+      </c>
+      <c r="E36" s="9" t="n">
+        <v>1196</v>
+      </c>
+      <c r="F36" s="9" t="n">
+        <v>290</v>
+      </c>
+      <c r="G36" s="10" t="n">
+        <v>0.2424749163879599</v>
+      </c>
+      <c r="H36" s="11" t="n">
+        <v>0.03147384415020621</v>
+      </c>
+      <c r="I36" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="J36" s="9" t="n">
+        <v>855</v>
+      </c>
+      <c r="K36" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="L36" s="8" t="inlineStr">
+        <is>
+          <t>2240043984</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n">
+        <v>722926</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>9788466243292</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>BRUJA MODERNA</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>196</v>
+      </c>
+      <c r="E37" s="9" t="n">
+        <v>1126</v>
+      </c>
+      <c r="F37" s="9" t="n">
+        <v>256</v>
+      </c>
+      <c r="G37" s="10" t="n">
+        <v>0.2273534635879219</v>
+      </c>
+      <c r="H37" s="11" t="n">
+        <v>0.0277838072498372</v>
+      </c>
+      <c r="I37" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="J37" s="9" t="n">
+        <v>811</v>
+      </c>
+      <c r="K37" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="L37" s="8" t="inlineStr">
+        <is>
+          <t>2240043558</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n">
+        <v>722861</v>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>9788466243063</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>ASTROCOACH</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>192</v>
+      </c>
+      <c r="E38" s="9" t="n">
+        <v>1038</v>
+      </c>
+      <c r="F38" s="9" t="n">
+        <v>183</v>
+      </c>
+      <c r="G38" s="10" t="n">
+        <v>0.1763005780346821</v>
+      </c>
+      <c r="H38" s="11" t="n">
+        <v>0.01986108096375081</v>
+      </c>
+      <c r="I38" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="J38" s="9" t="n">
+        <v>787</v>
+      </c>
+      <c r="K38" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="L38" s="8" t="inlineStr">
+        <is>
+          <t>2240043558</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n">
+        <v>734395</v>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>9789500216043</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>JUEGO Y APRENDO! DINOSAURIOS</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>192</v>
+      </c>
+      <c r="E39" s="9" t="n">
+        <v>1025</v>
+      </c>
+      <c r="F39" s="9" t="n">
+        <v>239</v>
+      </c>
+      <c r="G39" s="10" t="n">
+        <v>0.2331707317073171</v>
+      </c>
+      <c r="H39" s="11" t="n">
+        <v>0.0259387887996527</v>
+      </c>
+      <c r="I39" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="J39" s="9" t="n">
+        <v>767</v>
+      </c>
+      <c r="K39" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="L39" s="8" t="inlineStr">
+        <is>
+          <t>2240043779</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n">
+        <v>726373</v>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>9789500215350</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>APRENDO A LEER LAS LETRAS</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="n">
+        <v>187</v>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>989</v>
+      </c>
+      <c r="F40" s="9" t="n">
+        <v>287</v>
+      </c>
+      <c r="G40" s="10" t="n">
+        <v>0.2901921132457027</v>
+      </c>
+      <c r="H40" s="11" t="n">
+        <v>0.03114825265899718</v>
+      </c>
+      <c r="I40" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="J40" s="9" t="n">
+        <v>645</v>
+      </c>
+      <c r="K40" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="L40" s="8" t="inlineStr">
+        <is>
+          <t>2240043097 / 2240044025</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n">
+        <v>731835</v>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>9789500216036</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>ANIMALES CON SUPERPODERES</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="n">
+        <v>176</v>
+      </c>
+      <c r="E41" s="9" t="n">
+        <v>969</v>
+      </c>
+      <c r="F41" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G41" s="10" t="n">
+        <v>0.2342621259029928</v>
+      </c>
+      <c r="H41" s="11" t="n">
+        <v>0.02463642283481658</v>
+      </c>
+      <c r="I41" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="J41" s="9" t="n">
+        <v>688</v>
+      </c>
+      <c r="K41" s="8" t="n">
+        <v>68</v>
+      </c>
+      <c r="L41" s="8" t="inlineStr">
+        <is>
+          <t>2240043558</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n">
+        <v>726374</v>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>9789500215367</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>APRENDO A LEER LAS SILABAS</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>183</v>
+      </c>
+      <c r="E42" s="9" t="n">
+        <v>940</v>
+      </c>
+      <c r="F42" s="9" t="n">
+        <v>227</v>
+      </c>
+      <c r="G42" s="10" t="n">
+        <v>0.2414893617021276</v>
+      </c>
+      <c r="H42" s="11" t="n">
+        <v>0.02463642283481658</v>
+      </c>
+      <c r="I42" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="J42" s="9" t="n">
+        <v>665</v>
+      </c>
+      <c r="K42" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="L42" s="8" t="inlineStr">
+        <is>
+          <t>2240043097 / 2240044025</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n">
+        <v>737451</v>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>9789500216388</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>METAMORFOSIS, LA</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="n">
+        <v>168</v>
+      </c>
+      <c r="E43" s="9" t="n">
+        <v>928</v>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>278</v>
+      </c>
+      <c r="G43" s="10" t="n">
+        <v>0.2995689655172414</v>
+      </c>
+      <c r="H43" s="11" t="n">
+        <v>0.03017147818537009</v>
+      </c>
+      <c r="I43" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="J43" s="9" t="n">
+        <v>611</v>
+      </c>
+      <c r="K43" s="8" t="n">
+        <v>62</v>
+      </c>
+      <c r="L43" s="8" t="inlineStr">
+        <is>
+          <t>2240043984</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n">
+        <v>645284</v>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>9789500209144</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>BUHO HUGO, EL</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="n">
+        <v>181</v>
+      </c>
+      <c r="E44" s="9" t="n">
+        <v>925</v>
+      </c>
+      <c r="F44" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="G44" s="10" t="n">
+        <v>0.09513513513513513</v>
+      </c>
+      <c r="H44" s="11" t="n">
+        <v>0.009550683742131539</v>
+      </c>
+      <c r="I44" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="J44" s="9" t="n">
+        <v>817</v>
+      </c>
+      <c r="K44" s="8" t="n">
+        <v>127</v>
+      </c>
+      <c r="L44" s="8" t="inlineStr">
+        <is>
+          <t>2240044748</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n">
+        <v>645286</v>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>9789500209137</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>PANDA AMANDA, LA</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="n">
+        <v>174</v>
+      </c>
+      <c r="E45" s="9" t="n">
+        <v>899</v>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="G45" s="10" t="n">
+        <v>0.09788654060066741</v>
+      </c>
+      <c r="H45" s="11" t="n">
+        <v>0.009550683742131539</v>
+      </c>
+      <c r="I45" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="J45" s="9" t="n">
+        <v>787</v>
+      </c>
+      <c r="K45" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="L45" s="8" t="inlineStr">
+        <is>
+          <t>2240044748</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n">
+        <v>645289</v>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>9789500209120</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>GATITO TITO, EL</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>172</v>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>898</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>99</v>
+      </c>
+      <c r="G46" s="10" t="n">
+        <v>0.1102449888641425</v>
+      </c>
+      <c r="H46" s="11" t="n">
+        <v>0.01074451920989798</v>
+      </c>
+      <c r="I46" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="J46" s="9" t="n">
+        <v>779</v>
+      </c>
+      <c r="K46" s="8" t="n">
+        <v>115</v>
+      </c>
+      <c r="L46" s="8" t="inlineStr">
+        <is>
+          <t>2240044748</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="n">
+        <v>645291</v>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>9789500209113</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>RANA LILIANA, LA</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>173</v>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>893</v>
+      </c>
+      <c r="F47" s="9" t="n">
+        <v>112</v>
+      </c>
+      <c r="G47" s="10" t="n">
+        <v>0.1254199328107503</v>
+      </c>
+      <c r="H47" s="11" t="n">
+        <v>0.01215541567180378</v>
+      </c>
+      <c r="I47" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="J47" s="9" t="n">
+        <v>759</v>
+      </c>
+      <c r="K47" s="8" t="n">
+        <v>113</v>
+      </c>
+      <c r="L47" s="8" t="inlineStr">
+        <is>
+          <t>2240044748</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n">
+        <v>725694</v>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>9789500215312</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>ENIGMAS PARA DESCUBRIR HISTORIA MODERNA</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="n">
+        <v>164</v>
+      </c>
+      <c r="E48" s="9" t="n">
+        <v>884</v>
+      </c>
+      <c r="F48" s="9" t="n">
+        <v>182</v>
+      </c>
+      <c r="G48" s="10" t="n">
+        <v>0.2058823529411765</v>
+      </c>
+      <c r="H48" s="11" t="n">
+        <v>0.01975255046668114</v>
+      </c>
+      <c r="I48" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="J48" s="9" t="n">
+        <v>652</v>
+      </c>
+      <c r="K48" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="L48" s="8" t="inlineStr">
+        <is>
+          <t>2240043097</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="n">
+        <v>647070</v>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>9789500209359</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>MEJORES CUENTOS DE AMOR, LOS</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>172</v>
+      </c>
+      <c r="E49" s="9" t="n">
+        <v>859</v>
+      </c>
+      <c r="F49" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="G49" s="10" t="n">
+        <v>0.08265424912689173</v>
+      </c>
+      <c r="H49" s="11" t="n">
+        <v>0.007705665291947037</v>
+      </c>
+      <c r="I49" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="J49" s="9" t="n">
+        <v>745</v>
+      </c>
+      <c r="K49" s="8" t="n">
+        <v>117</v>
+      </c>
+      <c r="L49" s="8" t="inlineStr">
+        <is>
+          <t>2240043984</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n">
+        <v>740169</v>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>9788466244893</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>TAROT: CARTAS DE ADIVINACION, SABIDURIA Y AUTODESCUBRIMIENTO</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="n">
+        <v>133</v>
+      </c>
+      <c r="E50" s="9" t="n">
+        <v>838</v>
+      </c>
+      <c r="F50" s="9" t="n">
+        <v>245</v>
+      </c>
+      <c r="G50" s="10" t="n">
+        <v>0.2923627684964201</v>
+      </c>
+      <c r="H50" s="11" t="n">
+        <v>0.02658997178207076</v>
+      </c>
+      <c r="I50" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="J50" s="9" t="n">
+        <v>583</v>
+      </c>
+      <c r="K50" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="L50" s="8" t="inlineStr">
+        <is>
+          <t>2240045048</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="n">
+        <v>647074</v>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>9789500209342</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>MEJORES CUENTOS DE MISTERIO, LOS</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>163</v>
+      </c>
+      <c r="E51" s="9" t="n">
+        <v>838</v>
+      </c>
+      <c r="F51" s="9" t="n">
+        <v>101</v>
+      </c>
+      <c r="G51" s="10" t="n">
+        <v>0.1205250596658711</v>
+      </c>
+      <c r="H51" s="11" t="n">
+        <v>0.01096158020403733</v>
+      </c>
+      <c r="I51" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="J51" s="9" t="n">
+        <v>702</v>
+      </c>
+      <c r="K51" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="L51" s="8" t="inlineStr">
+        <is>
+          <t>2240043984</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n">
+        <v>725693</v>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>9789500215329</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>ENIGMAS PARA DESCUBRIR HISTORIA ANTIGUA</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="n">
+        <v>163</v>
+      </c>
+      <c r="E52" s="9" t="n">
+        <v>827</v>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>162</v>
+      </c>
+      <c r="G52" s="10" t="n">
+        <v>0.1958887545344619</v>
+      </c>
+      <c r="H52" s="11" t="n">
+        <v>0.01758194052528761</v>
+      </c>
+      <c r="I52" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="J52" s="9" t="n">
+        <v>617</v>
+      </c>
+      <c r="K52" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="L52" s="8" t="inlineStr">
+        <is>
+          <t>2240043097</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="n">
+        <v>647077</v>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>9789500209366</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>MEJORES CUENTOS DE TERROR, LOS</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="n">
+        <v>168</v>
+      </c>
+      <c r="E53" s="9" t="n">
+        <v>815</v>
+      </c>
+      <c r="F53" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="G53" s="10" t="n">
+        <v>0.105521472392638</v>
+      </c>
+      <c r="H53" s="11" t="n">
+        <v>0.009333622747992185</v>
+      </c>
+      <c r="I53" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="J53" s="9" t="n">
+        <v>705</v>
+      </c>
+      <c r="K53" s="8" t="n">
+        <v>113</v>
+      </c>
+      <c r="L53" s="8" t="inlineStr">
+        <is>
+          <t>2240043984</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="n">
+        <v>647075</v>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>9789500209304</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>GRAN GATSBY, EL</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="n">
+        <v>161</v>
+      </c>
+      <c r="E54" s="9" t="n">
+        <v>783</v>
+      </c>
+      <c r="F54" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="G54" s="10" t="n">
+        <v>0.1136653895274585</v>
+      </c>
+      <c r="H54" s="11" t="n">
+        <v>0.009659214239201215</v>
+      </c>
+      <c r="I54" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="J54" s="9" t="n">
+        <v>669</v>
+      </c>
+      <c r="K54" s="8" t="n">
+        <v>113</v>
+      </c>
+      <c r="L54" s="8" t="inlineStr">
+        <is>
+          <t>2240043984</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="n">
+        <v>742444</v>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>9789500216951</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>EXPLOREMOS LA CASA</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="n">
+        <v>145</v>
+      </c>
+      <c r="E55" s="9" t="n">
+        <v>778</v>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>107</v>
+      </c>
+      <c r="G55" s="10" t="n">
+        <v>0.1375321336760925</v>
+      </c>
+      <c r="H55" s="11" t="n">
+        <v>0.01161276318645539</v>
+      </c>
+      <c r="I55" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="J55" s="9" t="n">
+        <v>661</v>
+      </c>
+      <c r="K55" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="L55" s="8" t="inlineStr">
+        <is>
+          <t>2240044330</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n">
+        <v>647078</v>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>9789500209250</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>RETRATO DE DORIAN GRAY, EL</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="n">
+        <v>136</v>
+      </c>
+      <c r="E56" s="9" t="n">
+        <v>751</v>
+      </c>
+      <c r="F56" s="9" t="n">
+        <v>126</v>
+      </c>
+      <c r="G56" s="10" t="n">
+        <v>0.1677762982689747</v>
+      </c>
+      <c r="H56" s="11" t="n">
+        <v>0.01367484263077925</v>
+      </c>
+      <c r="I56" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="J56" s="9" t="n">
+        <v>595</v>
+      </c>
+      <c r="K56" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="L56" s="8" t="inlineStr">
+        <is>
+          <t>2240043984</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="n">
+        <v>647071</v>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>9789500209335</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>MEJORES CUENTOS FANTASTICOS, LOS</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="n">
+        <v>156</v>
+      </c>
+      <c r="E57" s="9" t="n">
+        <v>744</v>
+      </c>
+      <c r="F57" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G57" s="10" t="n">
+        <v>0.08870967741935484</v>
+      </c>
+      <c r="H57" s="11" t="n">
+        <v>0.007163012806598654</v>
+      </c>
+      <c r="I57" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="J57" s="9" t="n">
+        <v>638</v>
+      </c>
+      <c r="K57" s="8" t="n">
+        <v>114</v>
+      </c>
+      <c r="L57" s="8" t="inlineStr">
+        <is>
+          <t>2240043984</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n">
+        <v>734398</v>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>9789500216258</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>PASEO POR LA GRANJA</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E58" s="9" t="n">
+        <v>328</v>
+      </c>
+      <c r="F58" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="G58" s="10" t="n">
+        <v>0.1402439024390244</v>
+      </c>
+      <c r="H58" s="11" t="n">
+        <v>0.004992402865205123</v>
+      </c>
+      <c r="I58" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" s="9" t="n">
+        <v>282</v>
+      </c>
+      <c r="K58" s="8" t="n">
+        <v>59</v>
+      </c>
+      <c r="L58" s="8" t="inlineStr">
+        <is>
+          <t>2240043778</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="n">
+        <v>734399</v>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>9789500216241</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>PASEO POR LA PLAYA</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="E59" s="9" t="n">
+        <v>321</v>
+      </c>
+      <c r="F59" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="G59" s="10" t="n">
+        <v>0.1339563862928349</v>
+      </c>
+      <c r="H59" s="11" t="n">
+        <v>0.004666811373996093</v>
+      </c>
+      <c r="I59" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" s="9" t="n">
+        <v>277</v>
+      </c>
+      <c r="K59" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="L59" s="8" t="inlineStr">
+        <is>
+          <t>2240043778</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="n">
+        <v>737017</v>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>9789500216586</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>VINI, EL GUARDIAN DE LOS DESEOS</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E60" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F60" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="K60" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="L60" s="8" t="inlineStr">
+        <is>
+          <t>2240044024</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E61" s="14">
+        <f>SUM(E4:E60)</f>
+        <v/>
+      </c>
+      <c r="F61" s="14">
+        <f>SUM(F4:F60)</f>
+        <v/>
+      </c>
+      <c r="G61" s="4">
+        <f>F61/E61</f>
+        <v/>
+      </c>
+      <c r="I61" s="14">
+        <f>SUM(I4:I60)</f>
+        <v/>
+      </c>
+      <c r="J61" s="14">
+        <f>SUM(J4:J60)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:L60"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>